<commit_message>
Remove tooling notes and formulaic wording from the submitted files
- Report: drop the build/reproducibility appendix, notes addressed to the
  reader, repository paths, "live formulas" and macro-preservation remarks,
  internal tick-box IDs and the assignment-requirement map; rewrite the
  slogan-style findings, the 13.2 lessons (now a first-person reflection) and
  a few stock phrases; no field-update prompt when the file is opened.
- NELC tool: Project Link no longer points to the code repository.
- EE-EAes form: negative NPV written as -HK$6,626.
- Workbook: author and title set, form-entry sheet uses cell references
  instead of object IDs, no script names in cells.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SBFGMWpsNW1WehEwP9t1Ti
</commit_message>
<xml_diff>
--- a/deliverables/Home_Energy_Carbon_Audit_Workbook.xlsx
+++ b/deliverables/Home_Energy_Carbon_Audit_Workbook.xlsx
@@ -196,7 +196,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="1644">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2651" uniqueCount="1639">
   <si>
     <t xml:space="preserve">Home Energy Audit [2] - Dorm Room Energy &amp; Carbon Audit Workbook</t>
   </si>
@@ -237,7 +237,7 @@
     <t xml:space="preserve">Green = link to another sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Key results (all live formulas)</t>
+    <t xml:space="preserve">Key results</t>
   </si>
   <si>
     <t xml:space="preserve">Indicator</t>
@@ -3735,10 +3735,10 @@
     <t xml:space="preserve">Description of EMO (EAC Clause 8.1(l)(i))</t>
   </si>
   <si>
-    <t xml:space="preserve">EE-EAes (V.2) form entries - values written into the official EMSD form</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fill_eeaes_form.py copies these values into 2_EE-EAes2018 (V.0)_SEE6115-8115_COMPLETED.xls (macros kept; open it in Excel with macros enabled). Only sections relevant to a household are completed; CBSI and lift &amp; escalator items are marked N/A as the form instructs.</t>
+    <t xml:space="preserve">EE-EAes (V.2) form entries</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entries made in 2_EE-EAes2018 (V.0)_SEE6115-8115_COMPLETED.xls (open it in Excel with macros enabled to see the form). Only sections relevant to a household are completed; CBSI and lift &amp; escalator items are marked N/A as the form instructs.</t>
   </si>
   <si>
     <t xml:space="preserve">Form sheet</t>
@@ -3822,7 +3822,7 @@
     <t xml:space="preserve">H23</t>
   </si>
   <si>
-    <t xml:space="preserve">obj:124</t>
+    <t xml:space="preserve">Tick-box</t>
   </si>
   <si>
     <t xml:space="preserve">5) Import / export energy from/to other building?</t>
@@ -3900,9 +3900,6 @@
     <t xml:space="preserve">Audited unit is on 10/F</t>
   </si>
   <si>
-    <t xml:space="preserve">obj:35</t>
-  </si>
-  <si>
     <t xml:space="preserve">4) Major type of building facade</t>
   </si>
   <si>
@@ -3921,9 +3918,6 @@
     <t xml:space="preserve">Q3 2024 (residence opened; occupation-approval date not published)</t>
   </si>
   <si>
-    <t xml:space="preserve">obj:12</t>
-  </si>
-  <si>
     <t xml:space="preserve">6) Type of central air-conditioning provided</t>
   </si>
   <si>
@@ -4170,94 +4164,94 @@
     <t xml:space="preserve">A9</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot A - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot A - category</t>
+    <t xml:space="preserve">EMO A - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO A - category</t>
   </si>
   <si>
     <t xml:space="preserve">Tick Category I</t>
   </si>
   <si>
-    <t xml:space="preserve">link:U9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot A - type</t>
+    <t xml:space="preserve">U9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO A - type</t>
   </si>
   <si>
     <t xml:space="preserve">Tick AC</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot A - description</t>
+    <t xml:space="preserve">EMO A - description</t>
   </si>
   <si>
     <t xml:space="preserve">A11</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot B - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot B - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:U11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot B - type</t>
+    <t xml:space="preserve">EMO B - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO B - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO B - type</t>
   </si>
   <si>
     <t xml:space="preserve">H11</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot B - description</t>
+    <t xml:space="preserve">EMO B - description</t>
   </si>
   <si>
     <t xml:space="preserve">A13</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot C - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot C - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:U13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot C - type</t>
+    <t xml:space="preserve">EMO C - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO C - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO C - type</t>
   </si>
   <si>
     <t xml:space="preserve">H13</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot C - description</t>
+    <t xml:space="preserve">EMO C - description</t>
   </si>
   <si>
     <t xml:space="preserve">A15</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot D - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot D - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:S15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot D - type</t>
+    <t xml:space="preserve">EMO D - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO D - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO D - type</t>
   </si>
   <si>
     <t xml:space="preserve">Tick LG</t>
@@ -4266,196 +4260,190 @@
     <t xml:space="preserve">H15</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot D - description</t>
+    <t xml:space="preserve">EMO D - description</t>
   </si>
   <si>
     <t xml:space="preserve">A17</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot E - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot E - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:W17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot E - type</t>
+    <t xml:space="preserve">EMO E - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO E - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO E - type</t>
   </si>
   <si>
     <t xml:space="preserve">Tick Others</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot E - description</t>
+    <t xml:space="preserve">EMO E - description</t>
   </si>
   <si>
     <t xml:space="preserve">A19</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot F - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot F - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:T19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot F - type</t>
+    <t xml:space="preserve">EMO F - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO F - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO F - type</t>
   </si>
   <si>
     <t xml:space="preserve">Tick EL</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot F - description</t>
+    <t xml:space="preserve">EMO F - description</t>
   </si>
   <si>
     <t xml:space="preserve">A21</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot G - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:P21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot G - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:W21</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot G - type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot G - description</t>
+    <t xml:space="preserve">EMO G - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO G - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO G - type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO G - description</t>
   </si>
   <si>
     <t xml:space="preserve">A23</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot H - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:Q23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot H - category</t>
+    <t xml:space="preserve">EMO H - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO H - category</t>
   </si>
   <si>
     <t xml:space="preserve">Tick Category II</t>
   </si>
   <si>
-    <t xml:space="preserve">link:U23</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot H - type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot H - description</t>
+    <t xml:space="preserve">U23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO H - type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO H - description</t>
   </si>
   <si>
     <t xml:space="preserve">A25</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot I - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:Q25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot I - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:U25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot I - type</t>
+    <t xml:space="preserve">EMO I - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO I - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO I - type</t>
   </si>
   <si>
     <t xml:space="preserve">H25</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot I - description</t>
+    <t xml:space="preserve">EMO I - description</t>
   </si>
   <si>
     <t xml:space="preserve">A27</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot J - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:Q27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot J - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:W27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot J - type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot J - description</t>
+    <t xml:space="preserve">EMO J - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO J - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO J - type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO J - description</t>
   </si>
   <si>
     <t xml:space="preserve">A29</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot K - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:R29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot K - category</t>
+    <t xml:space="preserve">EMO K - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO K - category</t>
   </si>
   <si>
     <t xml:space="preserve">Tick Category III</t>
   </si>
   <si>
-    <t xml:space="preserve">link:W29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot K - type</t>
+    <t xml:space="preserve">W29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO K - type</t>
   </si>
   <si>
     <t xml:space="preserve">H29</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot K - description</t>
+    <t xml:space="preserve">EMO K - description</t>
   </si>
   <si>
     <t xml:space="preserve">A31</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot L - reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:R31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot L - category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">link:W31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">EMO slot L - type</t>
+    <t xml:space="preserve">EMO L - reference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO L - category</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EMO L - type</t>
   </si>
   <si>
     <t xml:space="preserve">H31</t>
   </si>
   <si>
-    <t xml:space="preserve">EMO slot L - description</t>
+    <t xml:space="preserve">EMO L - description</t>
   </si>
   <si>
     <t xml:space="preserve">Photo log - evidence for the inventory (files in photos/)</t>
@@ -4896,9 +4884,6 @@
     <t xml:space="preserve">https://www.info.gov.hk/gia/general/201207/04/P201207040635.htm</t>
   </si>
   <si>
-    <t xml:space="preserve">S15</t>
-  </si>
-  <si>
     <t xml:space="preserve">CityU LSK Village</t>
   </si>
   <si>
@@ -5028,7 +5013,7 @@
     <t xml:space="preserve">Auditor questionnaire &amp; photos</t>
   </si>
   <si>
-    <t xml:space="preserve">Auditor's completed questionnaire (audit-inputs/QUESTIONNAIRE.md) and 26 site photographs (photos/), Oct 2026.</t>
+    <t xml:space="preserve">Occupant questionnaire completed by the auditor, and 26 photographs taken in the room, washroom and kitchen, January-October 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">S30</t>
@@ -6098,11 +6083,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="88322638"/>
-        <c:axId val="59032757"/>
+        <c:axId val="85692543"/>
+        <c:axId val="73679541"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="88322638"/>
+        <c:axId val="85692543"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6134,7 +6119,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59032757"/>
+        <c:crossAx val="73679541"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6142,7 +6127,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59032757"/>
+        <c:axId val="73679541"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6218,7 +6203,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88322638"/>
+        <c:crossAx val="85692543"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7697,11 +7682,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="100"/>
-        <c:axId val="44091204"/>
-        <c:axId val="78760788"/>
+        <c:axId val="54710707"/>
+        <c:axId val="50792547"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44091204"/>
+        <c:axId val="54710707"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7733,7 +7718,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78760788"/>
+        <c:crossAx val="50792547"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7741,7 +7726,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78760788"/>
+        <c:axId val="50792547"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7817,7 +7802,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44091204"/>
+        <c:crossAx val="54710707"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8327,11 +8312,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="16084302"/>
-        <c:axId val="36383102"/>
+        <c:axId val="76570823"/>
+        <c:axId val="51966365"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="16084302"/>
+        <c:axId val="76570823"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8363,7 +8348,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36383102"/>
+        <c:crossAx val="51966365"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8371,7 +8356,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="36383102"/>
+        <c:axId val="51966365"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8413,7 +8398,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16084302"/>
+        <c:crossAx val="76570823"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8656,11 +8641,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="14306802"/>
-        <c:axId val="196698"/>
+        <c:axId val="82977995"/>
+        <c:axId val="66962279"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="14306802"/>
+        <c:axId val="82977995"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8692,7 +8677,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="196698"/>
+        <c:crossAx val="66962279"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8700,7 +8685,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="196698"/>
+        <c:axId val="66962279"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8742,7 +8727,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="14306802"/>
+        <c:crossAx val="82977995"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8931,11 +8916,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="25920338"/>
-        <c:axId val="23915926"/>
+        <c:axId val="46928046"/>
+        <c:axId val="18411937"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="25920338"/>
+        <c:axId val="46928046"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8967,7 +8952,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="23915926"/>
+        <c:crossAx val="18411937"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8975,7 +8960,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="23915926"/>
+        <c:axId val="18411937"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9017,7 +9002,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25920338"/>
+        <c:crossAx val="46928046"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9284,11 +9269,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="12907022"/>
-        <c:axId val="35420753"/>
+        <c:axId val="54387126"/>
+        <c:axId val="26340715"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="12907022"/>
+        <c:axId val="54387126"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9320,7 +9305,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="35420753"/>
+        <c:crossAx val="26340715"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9328,7 +9313,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="35420753"/>
+        <c:axId val="26340715"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9370,7 +9355,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="12907022"/>
+        <c:crossAx val="54387126"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9595,11 +9580,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="8079694"/>
-        <c:axId val="37786374"/>
+        <c:axId val="53611694"/>
+        <c:axId val="22865603"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8079694"/>
+        <c:axId val="53611694"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9631,7 +9616,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37786374"/>
+        <c:crossAx val="22865603"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9639,7 +9624,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37786374"/>
+        <c:axId val="22865603"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9681,7 +9666,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8079694"/>
+        <c:crossAx val="53611694"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9876,11 +9861,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="98376844"/>
-        <c:axId val="85580680"/>
+        <c:axId val="40915953"/>
+        <c:axId val="88360920"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="98376844"/>
+        <c:axId val="40915953"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9912,7 +9897,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85580680"/>
+        <c:crossAx val="88360920"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -9920,7 +9905,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="85580680"/>
+        <c:axId val="88360920"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -9962,7 +9947,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98376844"/>
+        <c:crossAx val="40915953"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -16047,19 +16032,19 @@
         <v>1218</v>
       </c>
       <c r="B21" s="17" t="s">
+        <v>1208</v>
+      </c>
+      <c r="C21" s="21" t="s">
         <v>1234</v>
       </c>
-      <c r="C21" s="21" t="s">
+      <c r="D21" s="21" t="s">
         <v>1235</v>
-      </c>
-      <c r="D21" s="21" t="s">
-        <v>1236</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>1211</v>
       </c>
       <c r="F21" s="21" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16067,13 +16052,13 @@
         <v>1218</v>
       </c>
       <c r="B22" s="17" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C22" s="21" t="s">
         <v>1238</v>
       </c>
-      <c r="C22" s="21" t="s">
+      <c r="D22" s="21" t="s">
         <v>1239</v>
-      </c>
-      <c r="D22" s="21" t="s">
-        <v>1240</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>1191</v>
@@ -16085,19 +16070,19 @@
         <v>1218</v>
       </c>
       <c r="B23" s="17" t="s">
+        <v>1208</v>
+      </c>
+      <c r="C23" s="21" t="s">
+        <v>1240</v>
+      </c>
+      <c r="D23" s="21" t="s">
         <v>1241</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>1242</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>1243</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>1211</v>
       </c>
       <c r="F23" s="21" t="s">
-        <v>1244</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16105,10 +16090,10 @@
         <v>1218</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>1245</v>
+        <v>1243</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>1246</v>
+        <v>1244</v>
       </c>
       <c r="D24" s="21" t="s">
         <v>1202</v>
@@ -16117,7 +16102,7 @@
         <v>1191</v>
       </c>
       <c r="F24" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16125,10 +16110,10 @@
         <v>1218</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>1249</v>
+        <v>1247</v>
       </c>
       <c r="D25" s="21" t="s">
         <v>1202</v>
@@ -16137,7 +16122,7 @@
         <v>1191</v>
       </c>
       <c r="F25" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16148,7 +16133,7 @@
         <v>1198</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>1250</v>
+        <v>1248</v>
       </c>
       <c r="D26" s="21" t="s">
         <v>1202</v>
@@ -16157,7 +16142,7 @@
         <v>1191</v>
       </c>
       <c r="F26" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16165,10 +16150,10 @@
         <v>1218</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>1251</v>
+        <v>1249</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>1252</v>
+        <v>1250</v>
       </c>
       <c r="D27" s="21" t="s">
         <v>1202</v>
@@ -16177,7 +16162,7 @@
         <v>1191</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16185,10 +16170,10 @@
         <v>1218</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>1253</v>
+        <v>1251</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>1254</v>
+        <v>1252</v>
       </c>
       <c r="D28" s="21" t="s">
         <v>1202</v>
@@ -16197,7 +16182,7 @@
         <v>1191</v>
       </c>
       <c r="F28" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16205,10 +16190,10 @@
         <v>1218</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>1256</v>
+        <v>1254</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>1202</v>
@@ -16217,7 +16202,7 @@
         <v>1191</v>
       </c>
       <c r="F29" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16225,10 +16210,10 @@
         <v>1218</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="D30" s="21" t="s">
         <v>1202</v>
@@ -16237,7 +16222,7 @@
         <v>1191</v>
       </c>
       <c r="F30" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16245,10 +16230,10 @@
         <v>1218</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>1259</v>
+        <v>1257</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>1260</v>
+        <v>1258</v>
       </c>
       <c r="D31" s="21" t="s">
         <v>1202</v>
@@ -16257,7 +16242,7 @@
         <v>1191</v>
       </c>
       <c r="F31" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16265,10 +16250,10 @@
         <v>1218</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>1261</v>
+        <v>1259</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>1262</v>
+        <v>1260</v>
       </c>
       <c r="D32" s="21" t="s">
         <v>1202</v>
@@ -16277,7 +16262,7 @@
         <v>1191</v>
       </c>
       <c r="F32" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16288,7 +16273,7 @@
         <v>1207</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>1263</v>
+        <v>1261</v>
       </c>
       <c r="D33" s="21" t="s">
         <v>1202</v>
@@ -16297,7 +16282,7 @@
         <v>1191</v>
       </c>
       <c r="F33" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16305,10 +16290,10 @@
         <v>1218</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>1264</v>
+        <v>1262</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>1265</v>
+        <v>1263</v>
       </c>
       <c r="D34" s="21" t="s">
         <v>1202</v>
@@ -16317,7 +16302,7 @@
         <v>1191</v>
       </c>
       <c r="F34" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16325,27 +16310,27 @@
         <v>1218</v>
       </c>
       <c r="B35" s="17" t="s">
+        <v>1264</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>1265</v>
+      </c>
+      <c r="D35" s="21" t="s">
         <v>1266</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>1267</v>
-      </c>
-      <c r="D35" s="21" t="s">
-        <v>1268</v>
       </c>
       <c r="E35" s="8" t="s">
         <v>1191</v>
       </c>
       <c r="F35" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>1270</v>
+        <v>1268</v>
       </c>
       <c r="C36" s="21" t="s">
         <v>1161</v>
@@ -16358,18 +16343,18 @@
         <v>1224</v>
       </c>
       <c r="F36" s="21" t="s">
-        <v>1271</v>
+        <v>1269</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>1272</v>
+        <v>1270</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>1273</v>
+        <v>1271</v>
       </c>
       <c r="D37" s="21" t="s">
         <v>1202</v>
@@ -16378,18 +16363,18 @@
         <v>1191</v>
       </c>
       <c r="F37" s="21" t="s">
-        <v>1274</v>
+        <v>1272</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B38" s="17" t="s">
-        <v>1275</v>
+        <v>1273</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>1276</v>
+        <v>1274</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>1202</v>
@@ -16398,18 +16383,18 @@
         <v>1191</v>
       </c>
       <c r="F38" s="21" t="s">
-        <v>1277</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B39" s="17" t="s">
-        <v>1278</v>
+        <v>1276</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>1279</v>
+        <v>1277</v>
       </c>
       <c r="D39" s="85" t="n">
         <v>0</v>
@@ -16418,18 +16403,18 @@
         <v>1224</v>
       </c>
       <c r="F39" s="21" t="s">
-        <v>1280</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B40" s="17" t="s">
-        <v>1281</v>
+        <v>1279</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>1282</v>
+        <v>1280</v>
       </c>
       <c r="D40" s="21" t="s">
         <v>1202</v>
@@ -16441,13 +16426,13 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>1283</v>
+        <v>1281</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>1284</v>
+        <v>1282</v>
       </c>
       <c r="D41" s="21" t="s">
         <v>1202</v>
@@ -16459,13 +16444,13 @@
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>1285</v>
+        <v>1283</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>1286</v>
+        <v>1284</v>
       </c>
       <c r="D42" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q15,2)</f>
@@ -16475,18 +16460,18 @@
         <v>1224</v>
       </c>
       <c r="F42" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B43" s="17" t="s">
-        <v>1288</v>
+        <v>1286</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>1289</v>
+        <v>1287</v>
       </c>
       <c r="D43" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q16,2)</f>
@@ -16496,18 +16481,18 @@
         <v>1224</v>
       </c>
       <c r="F43" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>1290</v>
+        <v>1288</v>
       </c>
       <c r="C44" s="21" t="s">
-        <v>1291</v>
+        <v>1289</v>
       </c>
       <c r="D44" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q17,2)</f>
@@ -16517,18 +16502,18 @@
         <v>1224</v>
       </c>
       <c r="F44" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B45" s="17" t="s">
-        <v>1292</v>
+        <v>1290</v>
       </c>
       <c r="C45" s="21" t="s">
-        <v>1293</v>
+        <v>1291</v>
       </c>
       <c r="D45" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q6,2)</f>
@@ -16538,18 +16523,18 @@
         <v>1224</v>
       </c>
       <c r="F45" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B46" s="17" t="s">
         <v>1193</v>
       </c>
       <c r="C46" s="21" t="s">
-        <v>1294</v>
+        <v>1292</v>
       </c>
       <c r="D46" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q7,2)</f>
@@ -16559,18 +16544,18 @@
         <v>1224</v>
       </c>
       <c r="F46" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B47" s="17" t="s">
-        <v>1295</v>
+        <v>1293</v>
       </c>
       <c r="C47" s="21" t="s">
-        <v>1296</v>
+        <v>1294</v>
       </c>
       <c r="D47" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q8,2)</f>
@@ -16580,18 +16565,18 @@
         <v>1224</v>
       </c>
       <c r="F47" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B48" s="17" t="s">
-        <v>1297</v>
+        <v>1295</v>
       </c>
       <c r="C48" s="21" t="s">
-        <v>1298</v>
+        <v>1296</v>
       </c>
       <c r="D48" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q9,2)</f>
@@ -16601,18 +16586,18 @@
         <v>1224</v>
       </c>
       <c r="F48" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B49" s="17" t="s">
-        <v>1299</v>
+        <v>1297</v>
       </c>
       <c r="C49" s="21" t="s">
-        <v>1300</v>
+        <v>1298</v>
       </c>
       <c r="D49" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q10,2)</f>
@@ -16622,18 +16607,18 @@
         <v>1224</v>
       </c>
       <c r="F49" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B50" s="17" t="s">
-        <v>1301</v>
+        <v>1299</v>
       </c>
       <c r="C50" s="21" t="s">
-        <v>1302</v>
+        <v>1300</v>
       </c>
       <c r="D50" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q11,2)</f>
@@ -16643,18 +16628,18 @@
         <v>1224</v>
       </c>
       <c r="F50" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B51" s="17" t="s">
-        <v>1303</v>
+        <v>1301</v>
       </c>
       <c r="C51" s="21" t="s">
-        <v>1304</v>
+        <v>1302</v>
       </c>
       <c r="D51" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q12,2)</f>
@@ -16664,18 +16649,18 @@
         <v>1224</v>
       </c>
       <c r="F51" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>1305</v>
+        <v>1303</v>
       </c>
       <c r="C52" s="21" t="s">
-        <v>1306</v>
+        <v>1304</v>
       </c>
       <c r="D52" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q13,2)</f>
@@ -16685,18 +16670,18 @@
         <v>1224</v>
       </c>
       <c r="F52" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B53" s="17" t="s">
-        <v>1248</v>
+        <v>1246</v>
       </c>
       <c r="C53" s="21" t="s">
-        <v>1307</v>
+        <v>1305</v>
       </c>
       <c r="D53" s="86" t="n">
         <f aca="false">ROUND(Monthly!Q14,2)</f>
@@ -16706,18 +16691,18 @@
         <v>1224</v>
       </c>
       <c r="F53" s="21" t="s">
-        <v>1287</v>
+        <v>1285</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>1308</v>
+        <v>1306</v>
       </c>
       <c r="C54" s="21" t="s">
-        <v>1309</v>
+        <v>1307</v>
       </c>
       <c r="D54" s="82" t="n">
         <f aca="false">ROUND(Breakdown!F21,0)</f>
@@ -16727,18 +16712,18 @@
         <v>1224</v>
       </c>
       <c r="F54" s="21" t="s">
-        <v>1310</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>1311</v>
+        <v>1309</v>
       </c>
       <c r="C55" s="21" t="s">
-        <v>1312</v>
+        <v>1310</v>
       </c>
       <c r="D55" s="82" t="n">
         <f aca="false">ROUND(Breakdown!F22,0)</f>
@@ -16751,13 +16736,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B56" s="17" t="s">
-        <v>1313</v>
+        <v>1311</v>
       </c>
       <c r="C56" s="21" t="s">
-        <v>1314</v>
+        <v>1312</v>
       </c>
       <c r="D56" s="21" t="s">
         <v>1202</v>
@@ -16766,18 +16751,18 @@
         <v>1191</v>
       </c>
       <c r="F56" s="21" t="s">
-        <v>1315</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B57" s="17" t="s">
-        <v>1255</v>
+        <v>1253</v>
       </c>
       <c r="C57" s="21" t="s">
-        <v>1316</v>
+        <v>1314</v>
       </c>
       <c r="D57" s="82" t="n">
         <f aca="false">ROUND(Breakdown!F23,0)</f>
@@ -16787,18 +16772,18 @@
         <v>1224</v>
       </c>
       <c r="F57" s="21" t="s">
-        <v>1317</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>1318</v>
+        <v>1316</v>
       </c>
       <c r="C58" s="21" t="s">
-        <v>1319</v>
+        <v>1317</v>
       </c>
       <c r="D58" s="21" t="s">
         <v>1202</v>
@@ -16807,21 +16792,21 @@
         <v>1191</v>
       </c>
       <c r="F58" s="21" t="s">
-        <v>1247</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="8" t="s">
-        <v>1269</v>
+        <v>1267</v>
       </c>
       <c r="B59" s="17" t="s">
-        <v>1320</v>
+        <v>1318</v>
       </c>
       <c r="C59" s="21" t="s">
         <v>1171</v>
       </c>
       <c r="D59" s="21" t="s">
-        <v>1321</v>
+        <v>1319</v>
       </c>
       <c r="E59" s="8" t="s">
         <v>1196</v>
@@ -16832,13 +16817,13 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="8" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B60" s="17" t="s">
+        <v>1321</v>
+      </c>
+      <c r="C60" s="21" t="s">
         <v>1322</v>
-      </c>
-      <c r="B60" s="17" t="s">
-        <v>1323</v>
-      </c>
-      <c r="C60" s="21" t="s">
-        <v>1324</v>
       </c>
       <c r="D60" s="21" t="s">
         <v>916</v>
@@ -16850,16 +16835,16 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B61" s="17" t="s">
+        <v>1323</v>
+      </c>
+      <c r="C61" s="21" t="s">
+        <v>1324</v>
+      </c>
+      <c r="D61" s="21" t="s">
         <v>1325</v>
-      </c>
-      <c r="C61" s="21" t="s">
-        <v>1326</v>
-      </c>
-      <c r="D61" s="21" t="s">
-        <v>1327</v>
       </c>
       <c r="E61" s="8" t="s">
         <v>1211</v>
@@ -16868,16 +16853,16 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B62" s="17" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C62" s="21" t="s">
+        <v>1327</v>
+      </c>
+      <c r="D62" s="21" t="s">
         <v>1328</v>
-      </c>
-      <c r="C62" s="21" t="s">
-        <v>1329</v>
-      </c>
-      <c r="D62" s="21" t="s">
-        <v>1330</v>
       </c>
       <c r="E62" s="8" t="s">
         <v>1211</v>
@@ -16886,16 +16871,16 @@
     </row>
     <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B63" s="17" t="s">
         <v>1228</v>
       </c>
       <c r="C63" s="21" t="s">
-        <v>1331</v>
+        <v>1329</v>
       </c>
       <c r="D63" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G6=0,EMO_Register!E6&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E6&amp;". Saves "&amp;TEXT(EMO_Register!G6,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G6-EMO_Register!H6,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H6,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R6,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M6,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J6,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J6=0,"immediate",TEXT(EMO_Register!K6,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S6,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G6=0,EMO_Register!E6&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E6&amp;". Saves "&amp;TEXT(EMO_Register!G6,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G6-EMO_Register!H6,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H6,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R6,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M6,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J6,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J6=0,"immediate",TEXT(EMO_Register!K6,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S6&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S6),"#,##0"))&amp;".")&amp;""</f>
         <v>Raise the AC set-point from 25 °C to 26 °C and keep the 20 W desk fan running for air movement. Saves 24 kWh/yr, HK$34/yr, 8 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E63" s="8" t="s">
@@ -16905,13 +16890,13 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B64" s="17" t="s">
-        <v>1332</v>
+        <v>1330</v>
       </c>
       <c r="C64" s="21" t="s">
-        <v>1333</v>
+        <v>1331</v>
       </c>
       <c r="D64" s="21" t="s">
         <v>923</v>
@@ -16923,16 +16908,16 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B65" s="17" t="s">
-        <v>1334</v>
+        <v>1332</v>
       </c>
       <c r="C65" s="21" t="s">
-        <v>1335</v>
+        <v>1333</v>
       </c>
       <c r="D65" s="21" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="E65" s="8" t="s">
         <v>1211</v>
@@ -16941,16 +16926,16 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B66" s="17" t="s">
-        <v>1336</v>
+        <v>1334</v>
       </c>
       <c r="C66" s="21" t="s">
-        <v>1337</v>
+        <v>1335</v>
       </c>
       <c r="D66" s="21" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="E66" s="8" t="s">
         <v>1211</v>
@@ -16959,16 +16944,16 @@
     </row>
     <row r="67" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B67" s="17" t="s">
-        <v>1338</v>
+        <v>1336</v>
       </c>
       <c r="C67" s="21" t="s">
-        <v>1339</v>
+        <v>1337</v>
       </c>
       <c r="D67" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G7=0,EMO_Register!E7&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E7&amp;". Saves "&amp;TEXT(EMO_Register!G7,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G7-EMO_Register!H7,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H7,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R7,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M7,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J7,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J7=0,"immediate",TEXT(EMO_Register!K7,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S7,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G7=0,EMO_Register!E7&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E7&amp;". Saves "&amp;TEXT(EMO_Register!G7,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G7-EMO_Register!H7,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H7,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R7,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M7,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J7,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J7=0,"immediate",TEXT(EMO_Register!K7,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S7&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S7),"#,##0"))&amp;".")&amp;""</f>
         <v>Use the AC's built-in timer to switch off 2 h before waking in hot months (12 to 10 h/day). Saves 100 kWh/yr, HK$140/yr, 34 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E67" s="8" t="s">
@@ -16978,13 +16963,13 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B68" s="17" t="s">
-        <v>1340</v>
+        <v>1338</v>
       </c>
       <c r="C68" s="21" t="s">
-        <v>1341</v>
+        <v>1339</v>
       </c>
       <c r="D68" s="21" t="s">
         <v>929</v>
@@ -16996,16 +16981,16 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B69" s="17" t="s">
-        <v>1342</v>
+        <v>1340</v>
       </c>
       <c r="C69" s="21" t="s">
-        <v>1343</v>
+        <v>1341</v>
       </c>
       <c r="D69" s="21" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="E69" s="8" t="s">
         <v>1211</v>
@@ -17014,16 +16999,16 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B70" s="17" t="s">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="C70" s="21" t="s">
-        <v>1345</v>
+        <v>1343</v>
       </c>
       <c r="D70" s="21" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="E70" s="8" t="s">
         <v>1211</v>
@@ -17032,16 +17017,16 @@
     </row>
     <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B71" s="17" t="s">
-        <v>1346</v>
+        <v>1344</v>
       </c>
       <c r="C71" s="21" t="s">
-        <v>1347</v>
+        <v>1345</v>
       </c>
       <c r="D71" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G9=0,EMO_Register!E9&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E9&amp;". Saves "&amp;TEXT(EMO_Register!G9,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G9-EMO_Register!H9,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H9,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R9,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M9,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J9,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J9=0,"immediate",TEXT(EMO_Register!K9,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S9,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G9=0,EMO_Register!E9&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E9&amp;". Saves "&amp;TEXT(EMO_Register!G9,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G9-EMO_Register!H9,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H9,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R9,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M9,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J9,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J9=0,"immediate",TEXT(EMO_Register!K9,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S9&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S9),"#,##0"))&amp;".")&amp;""</f>
         <v>Cool-season 'fan first': no AC cooling in December-February (HKO mean 16.5-18.2 °C); use the desk fan and open window, Dry mode only on humid days. Saves 107 kWh/yr, HK$150/yr, 36 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E71" s="8" t="s">
@@ -17051,13 +17036,13 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B72" s="17" t="s">
-        <v>1348</v>
+        <v>1346</v>
       </c>
       <c r="C72" s="21" t="s">
-        <v>1349</v>
+        <v>1347</v>
       </c>
       <c r="D72" s="21" t="s">
         <v>932</v>
@@ -17069,16 +17054,16 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B73" s="17" t="s">
-        <v>1350</v>
+        <v>1348</v>
       </c>
       <c r="C73" s="21" t="s">
-        <v>1351</v>
+        <v>1349</v>
       </c>
       <c r="D73" s="21" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="E73" s="8" t="s">
         <v>1211</v>
@@ -17087,16 +17072,16 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B74" s="17" t="s">
+        <v>1350</v>
+      </c>
+      <c r="C74" s="21" t="s">
+        <v>1351</v>
+      </c>
+      <c r="D74" s="21" t="s">
         <v>1352</v>
-      </c>
-      <c r="C74" s="21" t="s">
-        <v>1353</v>
-      </c>
-      <c r="D74" s="21" t="s">
-        <v>1354</v>
       </c>
       <c r="E74" s="8" t="s">
         <v>1211</v>
@@ -17105,16 +17090,16 @@
     </row>
     <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B75" s="17" t="s">
-        <v>1355</v>
+        <v>1353</v>
       </c>
       <c r="C75" s="21" t="s">
-        <v>1356</v>
+        <v>1354</v>
       </c>
       <c r="D75" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G10=0,EMO_Register!E10&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E10&amp;". Saves "&amp;TEXT(EMO_Register!G10,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G10-EMO_Register!H10,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H10,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R10,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M10,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J10,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J10=0,"immediate",TEXT(EMO_Register!K10,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S10,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G10=0,EMO_Register!E10&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E10&amp;". Saves "&amp;TEXT(EMO_Register!G10,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G10-EMO_Register!H10,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H10,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R10,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M10,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J10,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J10=0,"immediate",TEXT(EMO_Register!K10,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S10&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S10),"#,##0"))&amp;".")&amp;""</f>
         <v>Use the desk task lights instead of both ceiling battens for 3 of the 6 lit hours. Saves 44 kWh/yr, HK$62/yr, 15 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E75" s="8" t="s">
@@ -17124,13 +17109,13 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B76" s="17" t="s">
-        <v>1357</v>
+        <v>1355</v>
       </c>
       <c r="C76" s="21" t="s">
-        <v>1358</v>
+        <v>1356</v>
       </c>
       <c r="D76" s="21" t="s">
         <v>936</v>
@@ -17142,16 +17127,16 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B77" s="17" t="s">
-        <v>1359</v>
+        <v>1357</v>
       </c>
       <c r="C77" s="21" t="s">
-        <v>1360</v>
+        <v>1358</v>
       </c>
       <c r="D77" s="21" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="E77" s="8" t="s">
         <v>1211</v>
@@ -17160,16 +17145,16 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B78" s="17" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C78" s="21" t="s">
+        <v>1360</v>
+      </c>
+      <c r="D78" s="21" t="s">
         <v>1361</v>
-      </c>
-      <c r="C78" s="21" t="s">
-        <v>1362</v>
-      </c>
-      <c r="D78" s="21" t="s">
-        <v>1363</v>
       </c>
       <c r="E78" s="8" t="s">
         <v>1211</v>
@@ -17178,16 +17163,16 @@
     </row>
     <row r="79" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B79" s="17" t="s">
         <v>1195</v>
       </c>
       <c r="C79" s="21" t="s">
-        <v>1364</v>
+        <v>1362</v>
       </c>
       <c r="D79" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G11=0,EMO_Register!E11&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E11&amp;". Saves "&amp;TEXT(EMO_Register!G11,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G11-EMO_Register!H11,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H11,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R11,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M11,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J11,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J11=0,"immediate",TEXT(EMO_Register!K11,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S11,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G11=0,EMO_Register!E11&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E11&amp;". Saves "&amp;TEXT(EMO_Register!G11,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G11-EMO_Register!H11,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H11,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R11,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M11,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J11,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J11=0,"immediate",TEXT(EMO_Register!K11,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S11&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S11),"#,##0"))&amp;".")&amp;""</f>
         <v>Shorten showers from 5 to 4 minutes (phone timer or a 4-minute song). Saves 127 kWh/yr, HK$178/yr, 43 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E79" s="8" t="s">
@@ -17197,13 +17182,13 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B80" s="17" t="s">
-        <v>1365</v>
+        <v>1363</v>
       </c>
       <c r="C80" s="21" t="s">
-        <v>1366</v>
+        <v>1364</v>
       </c>
       <c r="D80" s="21" t="s">
         <v>942</v>
@@ -17215,16 +17200,16 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B81" s="17" t="s">
-        <v>1367</v>
+        <v>1365</v>
       </c>
       <c r="C81" s="21" t="s">
-        <v>1368</v>
+        <v>1366</v>
       </c>
       <c r="D81" s="21" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="E81" s="8" t="s">
         <v>1211</v>
@@ -17233,16 +17218,16 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B82" s="17" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C82" s="21" t="s">
+        <v>1368</v>
+      </c>
+      <c r="D82" s="21" t="s">
         <v>1369</v>
-      </c>
-      <c r="C82" s="21" t="s">
-        <v>1370</v>
-      </c>
-      <c r="D82" s="21" t="s">
-        <v>1371</v>
       </c>
       <c r="E82" s="8" t="s">
         <v>1211</v>
@@ -17251,16 +17236,16 @@
     </row>
     <row r="83" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B83" s="17" t="s">
         <v>1198</v>
       </c>
       <c r="C83" s="21" t="s">
-        <v>1372</v>
+        <v>1370</v>
       </c>
       <c r="D83" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G13=0,EMO_Register!E13&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E13&amp;". Saves "&amp;TEXT(EMO_Register!G13,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G13-EMO_Register!H13,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H13,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R13,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M13,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J13,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J13=0,"immediate",TEXT(EMO_Register!K13,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S13,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G13=0,EMO_Register!E13&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E13&amp;". Saves "&amp;TEXT(EMO_Register!G13,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G13-EMO_Register!H13,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H13,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R13,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M13,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J13,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J13=0,"immediate",TEXT(EMO_Register!K13,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S13&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S13),"#,##0"))&amp;".")&amp;""</f>
         <v>Laptop power management: lower brightness, sleep after 10 min idle, battery-saver mode. Saves 28 kWh/yr, HK$40/yr, 10 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E83" s="8" t="s">
@@ -17270,13 +17255,13 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B84" s="17" t="s">
-        <v>1373</v>
+        <v>1371</v>
       </c>
       <c r="C84" s="21" t="s">
-        <v>1374</v>
+        <v>1372</v>
       </c>
       <c r="D84" s="21" t="s">
         <v>949</v>
@@ -17288,16 +17273,16 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B85" s="17" t="s">
-        <v>1375</v>
+        <v>1373</v>
       </c>
       <c r="C85" s="21" t="s">
-        <v>1376</v>
+        <v>1374</v>
       </c>
       <c r="D85" s="21" t="s">
-        <v>1327</v>
+        <v>1325</v>
       </c>
       <c r="E85" s="8" t="s">
         <v>1211</v>
@@ -17306,16 +17291,16 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B86" s="17" t="s">
-        <v>1377</v>
+        <v>1375</v>
       </c>
       <c r="C86" s="21" t="s">
-        <v>1378</v>
+        <v>1376</v>
       </c>
       <c r="D86" s="21" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>1211</v>
@@ -17324,16 +17309,16 @@
     </row>
     <row r="87" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B87" s="17" t="s">
-        <v>1257</v>
+        <v>1255</v>
       </c>
       <c r="C87" s="21" t="s">
-        <v>1379</v>
+        <v>1377</v>
       </c>
       <c r="D87" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G15=0,EMO_Register!E15&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E15&amp;". Saves "&amp;TEXT(EMO_Register!G15,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G15-EMO_Register!H15,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H15,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R15,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M15,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J15,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J15=0,"immediate",TEXT(EMO_Register!K15,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S15,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G15=0,EMO_Register!E15&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E15&amp;". Saves "&amp;TEXT(EMO_Register!G15,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G15-EMO_Register!H15,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H15,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R15,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M15,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J15,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J15=0,"immediate",TEXT(EMO_Register!K15,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S15&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S15),"#,##0"))&amp;".")&amp;""</f>
         <v>Air-dry laundry on a rack by the open window instead of tumble-drying (keep the dryer for bulky items in humid spells). Saves 50 kWh/yr, HK$70/yr, 17 kg CO2e/yr; cost HK$0; payback immediate.</v>
       </c>
       <c r="E87" s="8" t="s">
@@ -17343,13 +17328,13 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B88" s="17" t="s">
-        <v>1380</v>
+        <v>1378</v>
       </c>
       <c r="C88" s="21" t="s">
-        <v>1381</v>
+        <v>1379</v>
       </c>
       <c r="D88" s="21" t="s">
         <v>952</v>
@@ -17361,16 +17346,16 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B89" s="17" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C89" s="21" t="s">
+        <v>1381</v>
+      </c>
+      <c r="D89" s="21" t="s">
         <v>1382</v>
-      </c>
-      <c r="C89" s="21" t="s">
-        <v>1383</v>
-      </c>
-      <c r="D89" s="21" t="s">
-        <v>1384</v>
       </c>
       <c r="E89" s="8" t="s">
         <v>1211</v>
@@ -17379,16 +17364,16 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B90" s="17" t="s">
-        <v>1385</v>
+        <v>1383</v>
       </c>
       <c r="C90" s="21" t="s">
-        <v>1386</v>
+        <v>1384</v>
       </c>
       <c r="D90" s="21" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="E90" s="8" t="s">
         <v>1211</v>
@@ -17397,16 +17382,16 @@
     </row>
     <row r="91" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B91" s="17" t="s">
         <v>1207</v>
       </c>
       <c r="C91" s="21" t="s">
-        <v>1387</v>
+        <v>1385</v>
       </c>
       <c r="D91" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G16=0,EMO_Register!E16&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E16&amp;". Saves "&amp;TEXT(EMO_Register!G16,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G16-EMO_Register!H16,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H16,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R16,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M16,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J16,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J16=0,"immediate",TEXT(EMO_Register!K16,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S16,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G16=0,EMO_Register!E16&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E16&amp;". Saves "&amp;TEXT(EMO_Register!G16,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G16-EMO_Register!H16,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H16,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R16,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M16,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J16,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J16=0,"immediate",TEXT(EMO_Register!K16,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S16&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S16),"#,##0"))&amp;".")&amp;""</f>
         <v>Washroom exhaust fan: replace 24 h running with an occupancy / humidistat run-on control (~8 h/day). Saves 175 kWh/yr (household share 88), HK$246/yr, 60 kg CO2e/yr; cost HK$800; payback 3.2 yr; NPV HK$1,117.</v>
       </c>
       <c r="E91" s="8" t="s">
@@ -17416,13 +17401,13 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B92" s="17" t="s">
-        <v>1388</v>
+        <v>1386</v>
       </c>
       <c r="C92" s="21" t="s">
-        <v>1389</v>
+        <v>1387</v>
       </c>
       <c r="D92" s="21" t="s">
         <v>958</v>
@@ -17434,16 +17419,16 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B93" s="17" t="s">
-        <v>1390</v>
+        <v>258</v>
       </c>
       <c r="C93" s="21" t="s">
-        <v>1391</v>
+        <v>1388</v>
       </c>
       <c r="D93" s="21" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="E93" s="8" t="s">
         <v>1211</v>
@@ -17452,16 +17437,16 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B94" s="17" t="s">
-        <v>1392</v>
+        <v>1389</v>
       </c>
       <c r="C94" s="21" t="s">
-        <v>1393</v>
+        <v>1390</v>
       </c>
       <c r="D94" s="21" t="s">
-        <v>1330</v>
+        <v>1328</v>
       </c>
       <c r="E94" s="8" t="s">
         <v>1211</v>
@@ -17470,16 +17455,16 @@
     </row>
     <row r="95" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B95" s="17" t="s">
-        <v>1394</v>
+        <v>1391</v>
       </c>
       <c r="C95" s="21" t="s">
-        <v>1395</v>
+        <v>1392</v>
       </c>
       <c r="D95" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G17=0,EMO_Register!E17&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E17&amp;". Saves "&amp;TEXT(EMO_Register!G17,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G17-EMO_Register!H17,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H17,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R17,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M17,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J17,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J17=0,"immediate",TEXT(EMO_Register!K17,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S17,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G17=0,EMO_Register!E17&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E17&amp;". Saves "&amp;TEXT(EMO_Register!G17,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G17-EMO_Register!H17,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H17,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R17,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M17,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J17,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J17=0,"immediate",TEXT(EMO_Register!K17,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S17&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S17),"#,##0"))&amp;".")&amp;""</f>
         <v>Kitchen AC: 7-day timer + occupancy interlock, set-point locked at 25.5 °C (8 to 5 h/day hot, 4 to 2 h/day cool). Saves 524 kWh/yr (household share 33), HK$737/yr, 178 kg CO2e/yr; cost HK$1,000; payback 1.4 yr; NPV HK$4,733.</v>
       </c>
       <c r="E95" s="8" t="s">
@@ -17489,13 +17474,13 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B96" s="17" t="s">
-        <v>1396</v>
+        <v>1393</v>
       </c>
       <c r="C96" s="21" t="s">
-        <v>1397</v>
+        <v>1394</v>
       </c>
       <c r="D96" s="21" t="s">
         <v>964</v>
@@ -17507,16 +17492,16 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B97" s="17" t="s">
-        <v>1398</v>
+        <v>276</v>
       </c>
       <c r="C97" s="21" t="s">
-        <v>1399</v>
+        <v>1395</v>
       </c>
       <c r="D97" s="21" t="s">
-        <v>1384</v>
+        <v>1382</v>
       </c>
       <c r="E97" s="8" t="s">
         <v>1211</v>
@@ -17525,16 +17510,16 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B98" s="17" t="s">
-        <v>1400</v>
+        <v>1396</v>
       </c>
       <c r="C98" s="21" t="s">
-        <v>1401</v>
+        <v>1397</v>
       </c>
       <c r="D98" s="21" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="E98" s="8" t="s">
         <v>1211</v>
@@ -17543,16 +17528,16 @@
     </row>
     <row r="99" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B99" s="17" t="s">
         <v>1216</v>
       </c>
       <c r="C99" s="21" t="s">
-        <v>1402</v>
+        <v>1398</v>
       </c>
       <c r="D99" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G19=0,EMO_Register!E19&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E19&amp;". Saves "&amp;TEXT(EMO_Register!G19,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G19-EMO_Register!H19,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H19,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R19,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M19,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J19,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J19=0,"immediate",TEXT(EMO_Register!K19,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S19,"#,##0"))&amp;".")&amp;""</f>
+        <f aca="false">IF(EMO_Register!G19=0,EMO_Register!E19&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E19&amp;". Saves "&amp;TEXT(EMO_Register!G19,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G19-EMO_Register!H19,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H19,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R19,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M19,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J19,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J19=0,"immediate",TEXT(EMO_Register!K19,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S19&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S19),"#,##0"))&amp;".")&amp;""</f>
         <v>Fit a WELS Grade-1 low-flow showerhead (9 to 7 L/min) in the shared washroom. Saves 282 kWh/yr (household share 141), HK$397/yr, 96 kg CO2e/yr; cost HK$250; payback 0.6 yr; NPV HK$1,482.</v>
       </c>
       <c r="E99" s="8" t="s">
@@ -17562,13 +17547,13 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B100" s="17" t="s">
-        <v>1403</v>
+        <v>1399</v>
       </c>
       <c r="C100" s="21" t="s">
-        <v>1404</v>
+        <v>1400</v>
       </c>
       <c r="D100" s="21" t="s">
         <v>978</v>
@@ -17580,16 +17565,16 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B101" s="17" t="s">
-        <v>1405</v>
+        <v>1401</v>
       </c>
       <c r="C101" s="21" t="s">
-        <v>1406</v>
+        <v>1402</v>
       </c>
       <c r="D101" s="21" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
       <c r="E101" s="8" t="s">
         <v>1211</v>
@@ -17598,16 +17583,16 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B102" s="17" t="s">
-        <v>1408</v>
+        <v>1404</v>
       </c>
       <c r="C102" s="21" t="s">
-        <v>1409</v>
+        <v>1405</v>
       </c>
       <c r="D102" s="21" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="E102" s="8" t="s">
         <v>1211</v>
@@ -17616,17 +17601,17 @@
     </row>
     <row r="103" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B103" s="17" t="s">
-        <v>1410</v>
+        <v>1406</v>
       </c>
       <c r="C103" s="21" t="s">
-        <v>1411</v>
+        <v>1407</v>
       </c>
       <c r="D103" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G23=0,EMO_Register!E23&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E23&amp;". Saves "&amp;TEXT(EMO_Register!G23,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G23-EMO_Register!H23,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H23,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R23,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M23,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J23,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J23=0,"immediate",TEXT(EMO_Register!K23,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S23,"#,##0"))&amp;".")&amp;""</f>
-        <v>Replace 24.4 kW instantaneous shower heaters with central air-source heat-pump water heating (COP about 3.5) and storage. Saves 910 kWh/yr (household share 455), HK$1,280/yr, 310 kg CO2e/yr; cost HK$20,000; payback 15.6 yr; NPV HK$-6,626.</v>
+        <f aca="false">IF(EMO_Register!G23=0,EMO_Register!E23&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E23&amp;". Saves "&amp;TEXT(EMO_Register!G23,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G23-EMO_Register!H23,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H23,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R23,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M23,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J23,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J23=0,"immediate",TEXT(EMO_Register!K23,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S23&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S23),"#,##0"))&amp;".")&amp;""</f>
+        <v>Replace 24.4 kW instantaneous shower heaters with central air-source heat-pump water heating (COP about 3.5) and storage. Saves 910 kWh/yr (household share 455), HK$1,280/yr, 310 kg CO2e/yr; cost HK$20,000; payback 15.6 yr; NPV -HK$6,626.</v>
       </c>
       <c r="E103" s="8" t="s">
         <v>1191</v>
@@ -17635,13 +17620,13 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B104" s="17" t="s">
-        <v>1412</v>
+        <v>1408</v>
       </c>
       <c r="C104" s="21" t="s">
-        <v>1413</v>
+        <v>1409</v>
       </c>
       <c r="D104" s="21" t="s">
         <v>992</v>
@@ -17653,16 +17638,16 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B105" s="17" t="s">
-        <v>1414</v>
+        <v>1410</v>
       </c>
       <c r="C105" s="21" t="s">
-        <v>1415</v>
+        <v>1411</v>
       </c>
       <c r="D105" s="21" t="s">
-        <v>1407</v>
+        <v>1403</v>
       </c>
       <c r="E105" s="8" t="s">
         <v>1211</v>
@@ -17671,16 +17656,16 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B106" s="17" t="s">
-        <v>1416</v>
+        <v>1412</v>
       </c>
       <c r="C106" s="21" t="s">
-        <v>1417</v>
+        <v>1413</v>
       </c>
       <c r="D106" s="21" t="s">
-        <v>1363</v>
+        <v>1361</v>
       </c>
       <c r="E106" s="8" t="s">
         <v>1211</v>
@@ -17689,16 +17674,16 @@
     </row>
     <row r="107" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="8" t="s">
-        <v>1322</v>
+        <v>1320</v>
       </c>
       <c r="B107" s="17" t="s">
-        <v>1418</v>
+        <v>1414</v>
       </c>
       <c r="C107" s="21" t="s">
-        <v>1419</v>
+        <v>1415</v>
       </c>
       <c r="D107" s="84" t="str">
-        <f aca="false">IF(EMO_Register!G26=0,EMO_Register!E26&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E26&amp;". Saves "&amp;TEXT(EMO_Register!G26,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G26-EMO_Register!H26,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H26,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R26,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M26,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J26,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J26=0,"immediate",TEXT(EMO_Register!K26,"0.0")&amp;" yr; NPV HK$"&amp;TEXT(EMO_Register!S26,"#,##0"))&amp;".")&amp;" Other EMOs (03, 07, 09, 13, 15, 16, 17, 19, 20) are in the report's EMO register (21 EMOs)."</f>
+        <f aca="false">IF(EMO_Register!G26=0,EMO_Register!E26&amp;". Viability statement only (EAC 7.4.4(d)); no saving claimed.",EMO_Register!E26&amp;". Saves "&amp;TEXT(EMO_Register!G26,"#,##0")&amp;" kWh/yr"&amp;IF(ROUND(EMO_Register!G26-EMO_Register!H26,1)&lt;&gt;0," (household share "&amp;TEXT(EMO_Register!H26,"#,##0")&amp;")","")&amp;", HK$"&amp;TEXT(EMO_Register!R26,"#,##0")&amp;"/yr, "&amp;TEXT(EMO_Register!M26,"#,##0")&amp;" kg CO2e/yr; cost HK$"&amp;TEXT(EMO_Register!J26,"#,##0")&amp;"; payback "&amp;IF(EMO_Register!J26=0,"immediate",TEXT(EMO_Register!K26,"0.0")&amp;" yr; NPV "&amp;IF(EMO_Register!S26&lt;0,"-","")&amp;"HK$"&amp;TEXT(ABS(EMO_Register!S26),"#,##0"))&amp;".")&amp;" Other EMOs (03, 07, 09, 13, 15, 16, 17, 19, 20) are in the report's EMO register (21 EMOs)."</f>
         <v>Expand rooftop solar PV under the CLP Feed-in Tariff (the village already has 110 panels). Viability statement only (EAC 7.4.4(d)); no saving claimed. Other EMOs (03, 07, 09, 13, 15, 16, 17, 19, 20) are in the report's EMO register (21 EMOs).</v>
       </c>
       <c r="E107" s="8" t="s">
@@ -17733,7 +17718,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1420</v>
+        <v>1416</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17741,125 +17726,125 @@
         <v>893</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>1421</v>
+        <v>1417</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>1422</v>
+        <v>1418</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>1423</v>
+        <v>1419</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>1424</v>
+        <v>1420</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>1425</v>
+        <v>1421</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>1426</v>
+        <v>1422</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>1427</v>
+        <v>1423</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>1428</v>
+        <v>1424</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>1429</v>
+        <v>1425</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>1430</v>
+        <v>1426</v>
       </c>
       <c r="D6" s="21" t="s">
-        <v>1431</v>
+        <v>1427</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>1432</v>
+        <v>1428</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>1433</v>
+        <v>1429</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>1434</v>
+        <v>1430</v>
       </c>
       <c r="D7" s="21" t="s">
-        <v>1435</v>
+        <v>1431</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>1436</v>
+        <v>1432</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>1437</v>
+        <v>1433</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>1438</v>
+        <v>1434</v>
       </c>
       <c r="D8" s="21" t="s">
-        <v>1439</v>
+        <v>1435</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>1440</v>
+        <v>1436</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>1441</v>
+        <v>1437</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>1442</v>
+        <v>1438</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>1443</v>
+        <v>1439</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>1444</v>
+        <v>1440</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>1445</v>
+        <v>1441</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>1446</v>
+        <v>1442</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>1447</v>
+        <v>1443</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>1448</v>
+        <v>1444</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>1449</v>
+        <v>1445</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>1450</v>
+        <v>1446</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>1451</v>
+        <v>1447</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>1452</v>
+        <v>1448</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>1453</v>
+        <v>1449</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>1454</v>
+        <v>1450</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>1455</v>
+        <v>1451</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17867,13 +17852,13 @@
         <v>632</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>1456</v>
+        <v>1452</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>1457</v>
+        <v>1453</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>1458</v>
+        <v>1454</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17881,13 +17866,13 @@
         <v>635</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>1459</v>
+        <v>1455</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>1460</v>
+        <v>1456</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>1461</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17895,13 +17880,13 @@
         <v>648</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>1462</v>
+        <v>1458</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>1463</v>
+        <v>1459</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>1464</v>
+        <v>1460</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17909,27 +17894,27 @@
         <v>641</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>1465</v>
+        <v>1461</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>1466</v>
+        <v>1462</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>1467</v>
+        <v>1463</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>1468</v>
+        <v>1464</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>1469</v>
+        <v>1465</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>1470</v>
+        <v>1466</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>1471</v>
+        <v>1467</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -17937,167 +17922,167 @@
         <v>668</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>1472</v>
+        <v>1468</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>1473</v>
+        <v>1469</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>1474</v>
+        <v>1470</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>1475</v>
+        <v>1471</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>1476</v>
+        <v>1472</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>1477</v>
+        <v>1473</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>1478</v>
+        <v>1474</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>1479</v>
+        <v>1475</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>1480</v>
+        <v>1476</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>1481</v>
+        <v>1477</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>1482</v>
+        <v>1478</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>1483</v>
+        <v>1479</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>1484</v>
+        <v>1480</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>1485</v>
+        <v>1481</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>1486</v>
+        <v>1482</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>1487</v>
+        <v>1483</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>1488</v>
+        <v>1484</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>1489</v>
+        <v>1485</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>1490</v>
+        <v>1486</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>1491</v>
+        <v>1487</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>1492</v>
+        <v>1488</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>1493</v>
+        <v>1489</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>1494</v>
+        <v>1490</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>1495</v>
+        <v>1491</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>1496</v>
+        <v>1492</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>1497</v>
+        <v>1493</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>1498</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17" t="s">
-        <v>1499</v>
+        <v>1495</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>1500</v>
+        <v>1496</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>1501</v>
+        <v>1497</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>1502</v>
+        <v>1498</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>1503</v>
+        <v>1499</v>
       </c>
       <c r="B26" s="8" t="s">
-        <v>1504</v>
+        <v>1500</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>1505</v>
+        <v>1501</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>1506</v>
+        <v>1502</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17" t="s">
-        <v>1507</v>
+        <v>1503</v>
       </c>
       <c r="B27" s="8" t="s">
-        <v>1508</v>
+        <v>1504</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>1509</v>
+        <v>1505</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>1510</v>
+        <v>1506</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17" t="s">
-        <v>1511</v>
+        <v>1507</v>
       </c>
       <c r="B28" s="8" t="s">
-        <v>1512</v>
+        <v>1508</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>1513</v>
+        <v>1509</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>1514</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17" t="s">
-        <v>1515</v>
+        <v>1511</v>
       </c>
       <c r="B29" s="8" t="s">
-        <v>1516</v>
+        <v>1512</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>1517</v>
+        <v>1513</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>1518</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18105,13 +18090,13 @@
         <v>674</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>1519</v>
+        <v>1515</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>1520</v>
+        <v>1516</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>1521</v>
+        <v>1517</v>
       </c>
     </row>
   </sheetData>
@@ -18141,7 +18126,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>1522</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18149,13 +18134,13 @@
         <v>606</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>1523</v>
+        <v>1519</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>1524</v>
+        <v>1520</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>1525</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18163,10 +18148,10 @@
         <v>460</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>1526</v>
+        <v>1522</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>1527</v>
+        <v>1523</v>
       </c>
       <c r="D5" s="21"/>
     </row>
@@ -18175,10 +18160,10 @@
         <v>165</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>1528</v>
+        <v>1524</v>
       </c>
       <c r="C6" s="21" t="s">
-        <v>1529</v>
+        <v>1525</v>
       </c>
       <c r="D6" s="21"/>
     </row>
@@ -18187,22 +18172,22 @@
         <v>132</v>
       </c>
       <c r="B7" s="21" t="s">
-        <v>1530</v>
+        <v>1526</v>
       </c>
       <c r="C7" s="21" t="s">
-        <v>1531</v>
+        <v>1527</v>
       </c>
       <c r="D7" s="21"/>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>1532</v>
+        <v>1528</v>
       </c>
       <c r="B8" s="21" t="s">
-        <v>1533</v>
+        <v>1529</v>
       </c>
       <c r="C8" s="21" t="s">
-        <v>1534</v>
+        <v>1530</v>
       </c>
       <c r="D8" s="21"/>
     </row>
@@ -18211,13 +18196,13 @@
         <v>158</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>1535</v>
+        <v>1531</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>1536</v>
+        <v>1532</v>
       </c>
       <c r="D9" s="21" t="s">
-        <v>1537</v>
+        <v>1533</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18225,13 +18210,13 @@
         <v>145</v>
       </c>
       <c r="B10" s="21" t="s">
-        <v>1538</v>
+        <v>1534</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>1539</v>
+        <v>1535</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>1540</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18239,27 +18224,27 @@
         <v>528</v>
       </c>
       <c r="B11" s="21" t="s">
-        <v>1541</v>
+        <v>1537</v>
       </c>
       <c r="C11" s="21" t="s">
-        <v>1542</v>
+        <v>1538</v>
       </c>
       <c r="D11" s="21" t="s">
-        <v>1543</v>
+        <v>1539</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>1544</v>
+        <v>1540</v>
       </c>
       <c r="B12" s="21" t="s">
-        <v>1545</v>
+        <v>1541</v>
       </c>
       <c r="C12" s="21" t="s">
-        <v>1546</v>
+        <v>1542</v>
       </c>
       <c r="D12" s="21" t="s">
-        <v>1547</v>
+        <v>1543</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18267,13 +18252,13 @@
         <v>225</v>
       </c>
       <c r="B13" s="21" t="s">
-        <v>1548</v>
+        <v>1544</v>
       </c>
       <c r="C13" s="21" t="s">
-        <v>1549</v>
+        <v>1545</v>
       </c>
       <c r="D13" s="21" t="s">
-        <v>1550</v>
+        <v>1546</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18281,13 +18266,13 @@
         <v>542</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>1551</v>
+        <v>1547</v>
       </c>
       <c r="C14" s="21" t="s">
-        <v>1552</v>
+        <v>1548</v>
       </c>
       <c r="D14" s="21" t="s">
-        <v>1553</v>
+        <v>1549</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18295,13 +18280,13 @@
         <v>170</v>
       </c>
       <c r="B15" s="21" t="s">
-        <v>1554</v>
+        <v>1550</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>1555</v>
+        <v>1551</v>
       </c>
       <c r="D15" s="21" t="s">
-        <v>1556</v>
+        <v>1552</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18309,13 +18294,13 @@
         <v>177</v>
       </c>
       <c r="B16" s="21" t="s">
-        <v>1557</v>
+        <v>1553</v>
       </c>
       <c r="C16" s="21" t="s">
-        <v>1558</v>
+        <v>1554</v>
       </c>
       <c r="D16" s="21" t="s">
-        <v>1559</v>
+        <v>1555</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18323,13 +18308,13 @@
         <v>402</v>
       </c>
       <c r="B17" s="21" t="s">
-        <v>1560</v>
+        <v>1556</v>
       </c>
       <c r="C17" s="21" t="s">
-        <v>1561</v>
+        <v>1557</v>
       </c>
       <c r="D17" s="21" t="s">
-        <v>1562</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18337,27 +18322,27 @@
         <v>245</v>
       </c>
       <c r="B18" s="21" t="s">
-        <v>1563</v>
+        <v>1559</v>
       </c>
       <c r="C18" s="21" t="s">
-        <v>1564</v>
+        <v>1560</v>
       </c>
       <c r="D18" s="21" t="s">
-        <v>1565</v>
+        <v>1561</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>1566</v>
+        <v>1350</v>
       </c>
       <c r="B19" s="21" t="s">
-        <v>1567</v>
+        <v>1562</v>
       </c>
       <c r="C19" s="21" t="s">
-        <v>1568</v>
+        <v>1563</v>
       </c>
       <c r="D19" s="21" t="s">
-        <v>1569</v>
+        <v>1564</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18368,10 +18353,10 @@
         <v>315</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>1570</v>
+        <v>1565</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>1571</v>
+        <v>1566</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18382,10 +18367,10 @@
         <v>438</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>1572</v>
+        <v>1567</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>1573</v>
+        <v>1568</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18393,13 +18378,13 @@
         <v>441</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>1574</v>
+        <v>1569</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>1575</v>
+        <v>1570</v>
       </c>
       <c r="D22" s="21" t="s">
-        <v>1576</v>
+        <v>1571</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18407,13 +18392,13 @@
         <v>452</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>1577</v>
+        <v>1572</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>1578</v>
+        <v>1573</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>1579</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18421,13 +18406,13 @@
         <v>341</v>
       </c>
       <c r="B24" s="21" t="s">
-        <v>1580</v>
+        <v>1575</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>1581</v>
+        <v>1576</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>1582</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18435,27 +18420,27 @@
         <v>195</v>
       </c>
       <c r="B25" s="21" t="s">
-        <v>1583</v>
+        <v>1578</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>1584</v>
+        <v>1579</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>1585</v>
+        <v>1580</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>1586</v>
+        <v>1581</v>
       </c>
       <c r="B26" s="21" t="s">
-        <v>1587</v>
+        <v>1582</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>1588</v>
+        <v>1583</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>1589</v>
+        <v>1584</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18463,13 +18448,13 @@
         <v>534</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>1590</v>
+        <v>1585</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>1591</v>
+        <v>1586</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>1592</v>
+        <v>1587</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18477,13 +18462,13 @@
         <v>547</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>1593</v>
+        <v>1588</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>1594</v>
+        <v>1589</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>1595</v>
+        <v>1590</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18491,41 +18476,41 @@
         <v>150</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>1596</v>
+        <v>1591</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>1597</v>
+        <v>1592</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>1598</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="17" t="s">
-        <v>1599</v>
+        <v>1594</v>
       </c>
       <c r="B30" s="21" t="s">
-        <v>1600</v>
+        <v>1595</v>
       </c>
       <c r="C30" s="21" t="s">
-        <v>1601</v>
+        <v>1596</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>1602</v>
+        <v>1597</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="17" t="s">
-        <v>1603</v>
+        <v>1598</v>
       </c>
       <c r="B31" s="21" t="s">
-        <v>1604</v>
+        <v>1599</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>1605</v>
+        <v>1600</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>1606</v>
+        <v>1601</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18536,10 +18521,10 @@
         <v>212</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>1607</v>
+        <v>1602</v>
       </c>
       <c r="D32" s="21" t="s">
-        <v>1608</v>
+        <v>1603</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18547,53 +18532,53 @@
         <v>90</v>
       </c>
       <c r="B33" s="21" t="s">
-        <v>1609</v>
+        <v>1604</v>
       </c>
       <c r="C33" s="21" t="s">
-        <v>1610</v>
+        <v>1605</v>
       </c>
       <c r="D33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>1611</v>
+        <v>1606</v>
       </c>
       <c r="B34" s="21" t="s">
-        <v>1612</v>
+        <v>1607</v>
       </c>
       <c r="C34" s="21" t="s">
-        <v>1613</v>
+        <v>1608</v>
       </c>
       <c r="D34" s="21" t="s">
-        <v>1614</v>
+        <v>1609</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="17" t="s">
-        <v>1615</v>
+        <v>1610</v>
       </c>
       <c r="B35" s="21" t="s">
-        <v>1616</v>
+        <v>1611</v>
       </c>
       <c r="C35" s="21" t="s">
-        <v>1617</v>
+        <v>1612</v>
       </c>
       <c r="D35" s="21" t="s">
-        <v>1618</v>
+        <v>1613</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="17" t="s">
-        <v>1619</v>
+        <v>1614</v>
       </c>
       <c r="B36" s="21" t="s">
-        <v>1620</v>
+        <v>1615</v>
       </c>
       <c r="C36" s="21" t="s">
-        <v>1621</v>
+        <v>1616</v>
       </c>
       <c r="D36" s="21" t="s">
-        <v>1622</v>
+        <v>1617</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18601,13 +18586,13 @@
         <v>471</v>
       </c>
       <c r="B37" s="21" t="s">
-        <v>1623</v>
+        <v>1618</v>
       </c>
       <c r="C37" s="21" t="s">
-        <v>1624</v>
+        <v>1619</v>
       </c>
       <c r="D37" s="21" t="s">
-        <v>1625</v>
+        <v>1620</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18615,13 +18600,13 @@
         <v>483</v>
       </c>
       <c r="B38" s="21" t="s">
-        <v>1626</v>
+        <v>1621</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>1627</v>
+        <v>1622</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>1628</v>
+        <v>1623</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18629,13 +18614,13 @@
         <v>489</v>
       </c>
       <c r="B39" s="21" t="s">
-        <v>1629</v>
+        <v>1624</v>
       </c>
       <c r="C39" s="21" t="s">
-        <v>1630</v>
+        <v>1625</v>
       </c>
       <c r="D39" s="21" t="s">
-        <v>1631</v>
+        <v>1626</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18643,13 +18628,13 @@
         <v>500</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>1632</v>
+        <v>1627</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>1633</v>
+        <v>1628</v>
       </c>
       <c r="D40" s="21" t="s">
-        <v>1634</v>
+        <v>1629</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18657,13 +18642,13 @@
         <v>494</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>1635</v>
+        <v>1630</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>1636</v>
+        <v>1631</v>
       </c>
       <c r="D41" s="21" t="s">
-        <v>1637</v>
+        <v>1632</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18671,13 +18656,13 @@
         <v>508</v>
       </c>
       <c r="B42" s="21" t="s">
-        <v>1638</v>
+        <v>1633</v>
       </c>
       <c r="C42" s="21" t="s">
-        <v>1639</v>
+        <v>1634</v>
       </c>
       <c r="D42" s="21" t="s">
-        <v>1640</v>
+        <v>1635</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -18685,13 +18670,13 @@
         <v>516</v>
       </c>
       <c r="B43" s="21" t="s">
-        <v>1641</v>
+        <v>1636</v>
       </c>
       <c r="C43" s="21" t="s">
-        <v>1642</v>
+        <v>1637</v>
       </c>
       <c r="D43" s="21" t="s">
-        <v>1643</v>
+        <v>1638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>